<commit_message>
Actualizar masivamente registros de PO a ' PO 2602-0711' en BD_Detalle_Tarimas
</commit_message>
<xml_diff>
--- a/BD_Detalle_Tarimas.xlsx
+++ b/BD_Detalle_Tarimas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,7 +474,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>PO: 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>PO-2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -8492,7 +8492,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -8796,7 +8796,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -8948,7 +8948,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -9328,7 +9328,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -9442,7 +9442,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -9860,7 +9860,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -10240,7 +10240,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -10316,7 +10316,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -10392,7 +10392,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -10430,7 +10430,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -10468,7 +10468,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -10772,7 +10772,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -11874,7 +11874,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11950,7 +11950,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -12026,7 +12026,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -12140,7 +12140,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12292,7 +12292,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -13470,7 +13470,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -13622,7 +13622,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -13698,7 +13698,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -13736,7 +13736,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -13926,7 +13926,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -13964,7 +13964,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -14078,7 +14078,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -14154,7 +14154,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -14192,7 +14192,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -14344,7 +14344,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>PO 2602-0711</t>
+          <t xml:space="preserve"> PO 2602-0711</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">

</xml_diff>

<commit_message>
Reparar base de datos y estandarizar 'Proyecto Interno' a formato INT-XXX. Habilitar autolimpieza en carga e importaciones
</commit_message>
<xml_diff>
--- a/BD_Detalle_Tarimas.xlsx
+++ b/BD_Detalle_Tarimas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4849,7 +4849,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -5229,7 +5229,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -5989,7 +5989,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -6103,7 +6103,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6369,7 +6369,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -6673,7 +6673,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -6711,7 +6711,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -6749,7 +6749,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -6863,7 +6863,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -6977,7 +6977,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -7205,7 +7205,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>INT-001</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>INT-004</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>INT-004</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -7319,7 +7319,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>INT-005</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>INT-006</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
@@ -7433,7 +7433,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
@@ -7471,7 +7471,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
@@ -7661,7 +7661,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
@@ -7699,7 +7699,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -7889,7 +7889,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>INT-002</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
@@ -8041,7 +8041,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -8117,7 +8117,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -8155,7 +8155,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
@@ -8231,7 +8231,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
@@ -8345,7 +8345,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
@@ -8383,7 +8383,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -8459,7 +8459,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
@@ -8497,7 +8497,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -8535,7 +8535,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -8573,7 +8573,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
@@ -8725,7 +8725,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
@@ -8839,7 +8839,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
@@ -9029,7 +9029,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -9257,7 +9257,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
@@ -9295,7 +9295,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -9409,7 +9409,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -9523,7 +9523,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -9599,7 +9599,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -9637,7 +9637,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -9713,7 +9713,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -9827,7 +9827,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -9865,7 +9865,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -10017,7 +10017,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>INT-008</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>INT-008</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -10093,7 +10093,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -10169,7 +10169,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -10283,7 +10283,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -10321,7 +10321,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -10435,7 +10435,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -10473,7 +10473,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -10587,7 +10587,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -10625,7 +10625,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -10701,7 +10701,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -10739,7 +10739,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -10777,7 +10777,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -10815,7 +10815,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -10853,7 +10853,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>INT-009</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -11043,7 +11043,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>INT-013</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>INT-012</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -11119,7 +11119,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -11157,7 +11157,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -11195,7 +11195,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -11233,7 +11233,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -11309,7 +11309,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -11347,7 +11347,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -11385,7 +11385,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -11461,7 +11461,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -11499,7 +11499,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -11537,7 +11537,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -11993,7 +11993,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
@@ -12031,7 +12031,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -12069,7 +12069,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -12145,7 +12145,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -12221,7 +12221,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
@@ -12297,7 +12297,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
@@ -12335,7 +12335,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -12411,7 +12411,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -12449,7 +12449,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -12487,7 +12487,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -12563,7 +12563,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -12601,7 +12601,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -12677,7 +12677,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -12715,7 +12715,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -12753,7 +12753,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -12791,7 +12791,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -12829,7 +12829,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -12905,7 +12905,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -13019,7 +13019,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
@@ -13057,7 +13057,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
@@ -13095,7 +13095,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
@@ -13133,7 +13133,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
@@ -13171,7 +13171,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>INT-007</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
@@ -13209,7 +13209,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>INT-015</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
@@ -13247,7 +13247,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>INT-015</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>INT-015</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
@@ -13323,7 +13323,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
@@ -13399,7 +13399,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -13437,7 +13437,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -13475,7 +13475,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -13665,7 +13665,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
@@ -13779,7 +13779,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
@@ -13817,7 +13817,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>INT-015</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
@@ -13969,7 +13969,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
@@ -14007,7 +14007,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -14045,7 +14045,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
@@ -14083,7 +14083,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>INT-003</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">

</xml_diff>

<commit_message>
Corregir registros del proyecto 'RECHASO' a 'Material Rechazado' e incluirlo en la autolimpieza de app.py
</commit_message>
<xml_diff>
--- a/BD_Detalle_Tarimas.xlsx
+++ b/BD_Detalle_Tarimas.xlsx
@@ -14653,7 +14653,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
@@ -14729,7 +14729,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -14767,7 +14767,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
@@ -14843,7 +14843,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
@@ -14919,7 +14919,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>RECHASO</t>
+          <t>Material Rechazado</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">

</xml_diff>

<commit_message>
Estandarizar todas las Ordenes de Compra (PO) al formato 'PO XXXX-XXXX' en bases de datos y app.py
</commit_message>
<xml_diff>
--- a/BD_Detalle_Tarimas.xlsx
+++ b/BD_Detalle_Tarimas.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PO-2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>PO-2603-2025</t>
+          <t>PO 2603-2025</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PO-2603-2077</t>
+          <t>PO 2603-2077</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>PO: 2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>PO: 2603-0711</t>
+          <t>PO 2603-0711</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>PO: 2603-0711</t>
+          <t>PO 2603-0711</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>PO: 2026-0619</t>
+          <t>PO 2026-0619</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>PO-2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -4882,7 +4882,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5224,7 +5224,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6212,7 +6212,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -6706,7 +6706,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -6972,7 +6972,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
@@ -7200,7 +7200,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2603-0771</t>
+          <t>PO 2603-0771</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2603-0771</t>
+          <t>PO 2603-0771</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>2603-0892</t>
+          <t>PO 2603-0892</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>2603-0939</t>
+          <t>PO 2603-0939</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -7656,7 +7656,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
@@ -7846,7 +7846,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -7960,7 +7960,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>2602-0482</t>
+          <t>PO 2602-0482</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
@@ -8036,7 +8036,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
@@ -8112,7 +8112,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -8150,7 +8150,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -8492,7 +8492,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -8796,7 +8796,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -8948,7 +8948,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -9100,7 +9100,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -9176,7 +9176,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -9328,7 +9328,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
@@ -9366,7 +9366,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -9442,7 +9442,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -9860,7 +9860,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
@@ -9974,7 +9974,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -10012,7 +10012,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>2603-1070</t>
+          <t>PO 2603-1070</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -10050,7 +10050,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2603-1070</t>
+          <t>PO 2603-1070</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -10088,7 +10088,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -10240,7 +10240,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
@@ -10316,7 +10316,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -10354,7 +10354,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -10392,7 +10392,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -10430,7 +10430,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -10468,7 +10468,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -10696,7 +10696,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
@@ -10772,7 +10772,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10962,7 +10962,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
@@ -11000,7 +11000,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>2603-1038</t>
+          <t>PO 2603-1038</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>2603-1329</t>
+          <t>PO 2603-1329</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>2603-1329</t>
+          <t>PO 2603-1329</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E283" t="inlineStr">
@@ -11190,7 +11190,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -11228,7 +11228,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E285" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E286" t="inlineStr">
@@ -11304,7 +11304,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11380,7 +11380,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -11456,7 +11456,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -11494,7 +11494,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -11532,7 +11532,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -11570,7 +11570,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11608,7 +11608,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -11684,7 +11684,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -11722,7 +11722,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11798,7 +11798,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -11836,7 +11836,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -11874,7 +11874,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -11950,7 +11950,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -12026,7 +12026,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -12140,7 +12140,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -12292,7 +12292,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -12406,7 +12406,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -12482,7 +12482,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -12520,7 +12520,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -12558,7 +12558,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -12596,7 +12596,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -12634,7 +12634,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -12672,7 +12672,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -12710,7 +12710,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -12748,7 +12748,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -12786,7 +12786,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -12824,7 +12824,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -12862,7 +12862,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -12900,7 +12900,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -12976,7 +12976,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -13014,7 +13014,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -13090,7 +13090,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -13128,7 +13128,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -13166,7 +13166,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>2603-0989</t>
+          <t>PO 2603-0989</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -13204,7 +13204,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>2603-1459</t>
+          <t>PO 2603-1459</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>2603-1459</t>
+          <t>PO 2603-1459</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -13280,7 +13280,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>2603-1459</t>
+          <t>PO 2603-1459</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -13432,7 +13432,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -13470,7 +13470,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -13546,7 +13546,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -13622,7 +13622,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -13698,7 +13698,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -13736,7 +13736,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -13850,7 +13850,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -13888,7 +13888,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>2603-1459</t>
+          <t>PO 2603-1459</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -13926,7 +13926,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -13964,7 +13964,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -14078,7 +14078,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -14154,7 +14154,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -14192,7 +14192,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -14230,7 +14230,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -14344,7 +14344,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PO 2602-0711</t>
+          <t>PO 2602-0711</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">

</xml_diff>